<commit_message>
Replace FlySky TX/RX with a custom ESP32 RC link
Swaps the stock FlySky transmitter/receiver pair for a self-written
dual-ESP32 link (ESP-NOW between an onboard RX ESP32 and a handheld
TX ESP32, with the RX generating a real SBUS output to the FC and a
failsafe watchdog), to demonstrate embedded programming alongside the
mechanical work. Updates the electrical architecture, BOM, weight
budget, manufacturing/assembly steps, requirements, test plan (RC-link
+ failsafe bench test), design journal, and resume/interview material
accordingly. Cost-neutral: new tier totals are Minimum ~$125 CAD,
Recommended ~$155 CAD, Maximum ~$281 CAD (previously ~$126/$156/$283).

Drone_Project_Guide.pdf and possibly Wiring_Diagram.pdf are now stale
and need manual regeneration; their source isn't in this repo.
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -1,17 +1,49 @@
 
-<file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
-  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
-  <sheets>
-    <sheet sheetId="1" name="BOM" state="visible" r:id="rId4"/>
-  </sheets>
-  <calcPr calcId="171027"/>
-</workbook>
+<file path=docProps\app.xml><?xml version="1.0" encoding="utf-8"?>
+<Properties xmlns="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:vt="http://schemas.openxmlformats.org/officeDocument/2006/docPropsVTypes">
+  <Application>Microsoft Excel</Application>
+  <DocSecurity>0</DocSecurity>
+  <ScaleCrop>false</ScaleCrop>
+  <HeadingPairs>
+    <vt:vector size="2" baseType="variant">
+      <vt:variant>
+        <vt:lpstr>Worksheets</vt:lpstr>
+      </vt:variant>
+      <vt:variant>
+        <vt:i4>1</vt:i4>
+      </vt:variant>
+    </vt:vector>
+  </HeadingPairs>
+  <TitlesOfParts>
+    <vt:vector size="1" baseType="lpstr">
+      <vt:lpstr>BOM</vt:lpstr>
+    </vt:vector>
+  </TitlesOfParts>
+  <Company/>
+  <Manager/>
+  <LinksUpToDate>false</LinksUpToDate>
+  <SharedDoc>false</SharedDoc>
+  <HyperlinksChanged>false</HyperlinksChanged>
+  <AppVersion>16.0300</AppVersion>
+</Properties>
 </file>
 
-<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="102">
+<file path=docProps\core.xml><?xml version="1.0" encoding="utf-8"?>
+<cp:coreProperties xmlns:cp="http://schemas.openxmlformats.org/package/2006/metadata/core-properties" xmlns:dc="http://purl.org/dc/elements/1.1/" xmlns:dcterms="http://purl.org/dc/terms/" xmlns:dcmitype="http://purl.org/dc/dcmitype/" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance">
+  <dc:creator>Unknown</dc:creator>
+  <dc:title/>
+  <dc:subject/>
+  <dc:description/>
+  <cp:keywords/>
+  <cp:category/>
+  <cp:lastModifiedBy>Unknown</cp:lastModifiedBy>
+  <dcterms:created xsi:type="dcterms:W3CDTF">2026-08-31T01:35:01Z</dcterms:created>
+  <dcterms:modified xsi:type="dcterms:W3CDTF">2026-08-31T01:35:01Z</dcterms:modified>
+</cp:coreProperties>
+</file>
+
+<file path=xl\sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="103">
   <si>
     <t>Category</t>
   </si>
@@ -79,43 +111,43 @@
     <t>Manufacturer-specified</t>
   </si>
   <si>
-    <t>Receiver/transmitter</t>
-  </si>
-  <si>
-    <t>FlySky FS-A8S receiver</t>
-  </si>
-  <si>
-    <t>2.4GHz 8CH, PPM/i-BUS/SBUS output</t>
-  </si>
-  <si>
-    <t>FlexRC</t>
-  </si>
-  <si>
-    <t>https://flexrc.com/product/flysky-fs-a8s-receiver/</t>
+    <t>RC link</t>
+  </si>
+  <si>
+    <t>ESP32-C3 Super Mini (onboard RX)</t>
+  </si>
+  <si>
+    <t>RISC-V, 2.4GHz WiFi, custom firmware: ESP-NOW RX -&gt; SBUS out (inverted UART) to FC</t>
+  </si>
+  <si>
+    <t>AliExpress</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005005319963906.html</t>
   </si>
   <si>
     <t>CHECK INVENTORY</t>
   </si>
   <si>
-    <t>FlySky-compatible transmitter (FS-i6 class)</t>
-  </si>
-  <si>
-    <t>2.4GHz AFHDS 2A handheld TX</t>
-  </si>
-  <si>
-    <t>University/already owned (est. $40-50 CAD if purchased new)</t>
+    <t>ESP32-WROOM-32 DevKit (handheld TX) + KY-023 dual-axis joystick x2 + momentary/toggle switch x2</t>
+  </si>
+  <si>
+    <t>Dual-core, 2.4GHz WiFi, custom firmware: reads sticks/switches -&gt; ESP-NOW out. 4 stick axes (throttle, yaw, pitch, roll) + 2 AUX switches (arm, payload release). Powered via USB power bank, already owned, not priced separately.</t>
+  </si>
+  <si>
+    <t>AliExpress (DevKit $2.20 + 2x joystick $0.60 + 2x switch ~$0.50 est.)</t>
   </si>
   <si>
     <t/>
   </si>
   <si>
-    <t>UNIVERSITY / CHECK INVENTORY</t>
-  </si>
-  <si>
-    <t>University</t>
-  </si>
-  <si>
-    <t>Estimated - not counted toward purchase budget per brief instruction</t>
+    <t>No</t>
+  </si>
+  <si>
+    <t>Purchased</t>
+  </si>
+  <si>
+    <t>Estimated - DevKit and joystick prices from real AliExpress listings found this session; switch price is a typical-component estimate, no specific listing checked</t>
   </si>
   <si>
     <t>Motors</t>
@@ -217,7 +249,7 @@
     <t>3D-printing material</t>
   </si>
   <si>
-    <t>PETG filament (frame + payload mechanism, ~15-20g)</t>
+    <t>PETG filament (frame + payload mechanism + TX enclosure, ~20-30g)</t>
   </si>
   <si>
     <t>Partial spool usage</t>
@@ -317,11 +349,14 @@
   </si>
   <si>
     <t>Note: USD-&gt;CAD at 1 USD = 1.39 CAD (2026-08-30). "University Available?" = CHECK INVENTORY items are shown at their real purchase price above but should be excluded from your actual out-of-pocket cost if available through U of C inventory. Minimum tier substitutes brushed motors + a brushed AIO FC for the Recommended tier's brushless motors + FC/ESC, per Electrical_Architecture.md; it cannot meet the 20-100g payload target.</t>
+  </si>
+  <si>
+    <t>Estimated - real AliExpress listings found this session, $3.50-4.80 USD range</t>
   </si>
 </sst>
 </file>
 
-<file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0.00"/>
@@ -387,7 +422,7 @@
 </styleSheet>
 </file>
 
-<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\theme\theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
@@ -707,7 +742,18 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl\workbook.xml><?xml version="1.0" encoding="utf-8"?>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
+  <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
+  <sheets>
+    <sheet sheetId="1" name="BOM" state="visible" r:id="rId4"/>
+  </sheets>
+  <calcPr calcId="171027"/>
+</workbook>
+</file>
+
+<file path=xl\worksheets\sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:L24"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -816,7 +862,7 @@
         <v>24</v>
       </c>
       <c r="E3" s="1">
-        <v>13.89</v>
+        <v>5.55</v>
       </c>
       <c r="F3" t="s">
         <v>25</v>
@@ -825,7 +871,7 @@
         <v>26</v>
       </c>
       <c r="H3" t="s">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="I3" t="s">
         <v>18</v>
@@ -837,7 +883,7 @@
         <v>20</v>
       </c>
       <c r="L3" t="s">
-        <v>21</v>
+        <v>102</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -854,7 +900,7 @@
         <v>29</v>
       </c>
       <c r="E4" s="1">
-        <v>0</v>
+        <v>6.12</v>
       </c>
       <c r="F4" t="s">
         <v>30</v>
@@ -1158,7 +1204,7 @@
         <v>69</v>
       </c>
       <c r="E12" s="1">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F12" t="s">
         <v>70</v>
@@ -1415,7 +1461,7 @@
         <v>98</v>
       </c>
       <c r="E20" s="5">
-        <v>125.9</v>
+        <v>124.68</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1423,7 +1469,7 @@
         <v>99</v>
       </c>
       <c r="E21" s="5">
-        <v>156.47</v>
+        <v>155.25</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1431,7 +1477,7 @@
         <v>100</v>
       </c>
       <c r="E22" s="5">
-        <v>282.68</v>
+        <v>281.46</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Switch motor source to cheaper AliExpress SPARKHOBBY 1103 11000KV listing
Replaces the Pyrodrone/BetaFPV 1103 11000KV motor ($50.99 USD/4-pack)
with a verified same-spec AliExpress listing (SPARKHOBBY XSPEED 1103
11000KV, 2-3S, 1.5mm shaft, Gemfan/HQprop 65mm compatible) at C$33.58
for 4, found after comparison-shopping several competing listings and
weeding out misleading multi-pack pricing.

Drops the Recommended-tier build cost from ~$155.25 CAD to ~$117.95
CAD (Maximum tier: ~$281.46 -> ~$206.86), bringing it much closer to
the original $100 CAD target. Updated bom_data.js (source of truth),
regenerated BOM.xlsx/Drone_Project_Guide.pdf/Wiring_Diagram.pdf, and
synced the cost narrative across README, Requirements, Design_Journal,
Electrical_Architecture, and Interview_Talking_Points.
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -112,16 +112,19 @@
     <t>Motors</t>
   </si>
   <si>
-    <t>1103 11000KV brushless motor (4-pack)</t>
-  </si>
-  <si>
-    <t>~3.3-3.55g each, 2S-rated, 1.5mm shaft, price is for the full set of 4</t>
-  </si>
-  <si>
-    <t>Pyrodrone (BetaFPV)</t>
-  </si>
-  <si>
-    <t>https://pyrodrone.com/products/betafpv-1103-11000kv-2s-brushless-motor-4pcs</t>
+    <t>SPARKHOBBY XSPEED 1103 11000KV brushless motor (4-pack)</t>
+  </si>
+  <si>
+    <t>2-3S rated, 1.5mm shaft, explicitly compatible with Gemfan/HQprop 65mm props; price is for the full set of 4; bare pigtail wire leads, no connector</t>
+  </si>
+  <si>
+    <t>AliExpress (Sparkhobby Store)</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005004927233900.html</t>
+  </si>
+  <si>
+    <t>Manufacturer-specified (price/specs from listing); per-motor weight not published on this specific listing, ~3.3-3.55g/motor is a cross-shopping Estimate from other 1103 11000KV listings, not confirmed for this product</t>
   </si>
   <si>
     <t>Propellers</t>
@@ -268,13 +271,10 @@
     <t>Spare/replacement</t>
   </si>
   <si>
-    <t>Spare motor set (4x 1103 11000KV)</t>
-  </si>
-  <si>
-    <t>Crash spares</t>
-  </si>
-  <si>
-    <t>Pyrodrone</t>
+    <t>Spare motor set (4x Sparkhobby XSPEED 1103 11000KV)</t>
+  </si>
+  <si>
+    <t>Crash spares, same listing as primary motor set</t>
   </si>
   <si>
     <t>Maximum</t>
@@ -889,7 +889,7 @@
         <v>34</v>
       </c>
       <c r="E5" s="1">
-        <v>70.88</v>
+        <v>33.58</v>
       </c>
       <c r="F5" t="s">
         <v>35</v>
@@ -910,30 +910,30 @@
         <v>20</v>
       </c>
       <c r="L5" t="s">
-        <v>21</v>
+        <v>37</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E6" s="1">
         <v>6.24</v>
       </c>
       <c r="F6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H6" t="s">
         <v>17</v>
@@ -953,28 +953,28 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="B7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E7" s="1">
         <v>8.33</v>
       </c>
       <c r="F7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="G7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="H7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I7" t="s">
         <v>18</v>
@@ -986,30 +986,30 @@
         <v>20</v>
       </c>
       <c r="L7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E8" s="1">
         <v>4.17</v>
       </c>
       <c r="F8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="H8" t="s">
         <v>17</v>
@@ -1029,25 +1029,25 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E9" s="1">
         <v>6</v>
       </c>
       <c r="F9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H9" t="s">
         <v>17</v>
@@ -1062,30 +1062,30 @@
         <v>20</v>
       </c>
       <c r="L9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="B10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E10" s="1">
         <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H10" t="s">
         <v>17</v>
@@ -1100,33 +1100,33 @@
         <v>20</v>
       </c>
       <c r="L10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E11" s="1">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H11" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I11" t="s">
         <v>18</v>
@@ -1138,33 +1138,33 @@
         <v>20</v>
       </c>
       <c r="L11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E12" s="1">
         <v>4</v>
       </c>
       <c r="F12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H12" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I12" t="s">
         <v>18</v>
@@ -1173,80 +1173,80 @@
         <v>19</v>
       </c>
       <c r="K12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="L12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="B13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E13" s="1">
         <v>12.51</v>
       </c>
       <c r="F13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H13" t="s">
         <v>17</v>
       </c>
       <c r="I13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K13" t="s">
         <v>20</v>
       </c>
       <c r="L13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E14" s="1">
         <v>59.76</v>
       </c>
       <c r="F14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="G14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="H14" t="s">
         <v>17</v>
       </c>
       <c r="I14" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="J14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="K14" t="s">
         <v>20</v>
@@ -1257,22 +1257,22 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E15" s="1">
-        <v>70.88</v>
+        <v>33.58</v>
       </c>
       <c r="F15" t="s">
-        <v>87</v>
+        <v>35</v>
       </c>
       <c r="G15" t="s">
         <v>36</v>
@@ -1295,7 +1295,7 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B16" t="s">
         <v>89</v>
@@ -1313,7 +1313,7 @@
         <v>91</v>
       </c>
       <c r="G16" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H16" t="s">
         <v>17</v>
@@ -1348,13 +1348,13 @@
         <v>12</v>
       </c>
       <c r="F17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H17" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I17" t="s">
         <v>17</v>
@@ -1366,7 +1366,7 @@
         <v>20</v>
       </c>
       <c r="L17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
@@ -1386,13 +1386,13 @@
         <v>35</v>
       </c>
       <c r="F18" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H18" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="I18" t="s">
         <v>17</v>
@@ -1404,7 +1404,7 @@
         <v>20</v>
       </c>
       <c r="L18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1420,7 +1420,7 @@
         <v>98</v>
       </c>
       <c r="E21" s="5">
-        <v>155.25</v>
+        <v>117.95</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
@@ -1428,7 +1428,7 @@
         <v>99</v>
       </c>
       <c r="E22" s="5">
-        <v>281.46</v>
+        <v>206.86</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Clean up leftover assistant-voice phrasing in docs and report
Reworded a handful of third-person/tool-call-sounding phrases left
over from earlier drafting passes so the documentation reads
consistently in first person: "the user has indicated" -> "I have",
references to "the brief's Section X" -> the actual doc name and
section, "found this session" / "fetch failed" / "live web search"
reworded to plain sourcing language, and "not independently
re-verified this session" -> "not independently re-verified yet".
Regenerated Drone_Project_Guide.pdf and BOM.xlsx to match.
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -91,7 +91,7 @@
     <t>https://www.aliexpress.com/item/1005005319963906.html</t>
   </si>
   <si>
-    <t>Estimated - real AliExpress listings found this session, $3.50-4.80 USD range</t>
+    <t>Estimated - real AliExpress listings found, $3.50-4.80 USD range</t>
   </si>
   <si>
     <t>ESP32-WROOM-32 DevKit (handheld TX) + KY-023 dual-axis joystick x2 + momentary/toggle switch x2</t>
@@ -106,7 +106,7 @@
     <t>https://www.aliexpress.com/item/1005003145871431.html ; https://www.aliexpress.com/item/1882818018.html</t>
   </si>
   <si>
-    <t>Estimated - DevKit and joystick prices from real AliExpress listings found this session; switch price is a typical-component estimate, no specific listing checked</t>
+    <t>Estimated - DevKit and joystick prices from real AliExpress listings found; switch price is a typical-component estimate, no specific listing checked</t>
   </si>
   <si>
     <t>Motors</t>
@@ -250,7 +250,7 @@
     <t>Minimum</t>
   </si>
   <si>
-    <t>Estimated (fetch failed, price not independently confirmed)</t>
+    <t>Estimated (price not independently confirmed)</t>
   </si>
   <si>
     <t>Flight controller (Minimum tier alt.)</t>

</xml_diff>

<commit_message>
Switch RC-link ESP32 boards to cheaper verified AliExpress listings
Replaces the RX (ESP32-C3 Super Mini, ~3.50-4.80 USD estimate) and TX
(ESP32-WROOM-32 DevKit, 2.20 USD estimate) with two verified listings:
ESP32-C3 Super Mini 4MB flash (C$1.68, 590 reviews/10,000+ sold,
Simple Robot Store) and ESP32-WROOM-32 DevKitC (C$1.40, 4.9 stars/32
reviews). Combined RX+TX cost drops from ~$11.67 CAD to ~$6.14 CAD.

Drops the Recommended-tier total from ~$117.95 CAD to ~$112.42 CAD
(Minimum: ~$124.68 -> ~$119.15, Maximum: ~$206.86 -> ~$201.33), since
the Minimum/Maximum tiers use the same RC link. Flagged in bom_data.js
that a minority of RX board reviews report WiFi not working out of
the box, worth bench-testing early per Test 5. Regenerated
BOM.xlsx/Drone_Project_Guide.pdf/Wiring_Diagram.pdf and synced the
cost narrative across README, Requirements, Design_Journal, and
Electrical_Architecture.
</commit_message>
<xml_diff>
--- a/BOM/BOM.xlsx
+++ b/BOM/BOM.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="101">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="102">
   <si>
     <t>Category</t>
   </si>
@@ -82,31 +82,34 @@
     <t>RC link</t>
   </si>
   <si>
-    <t>ESP32-C3 Super Mini (onboard RX)</t>
+    <t>ESP32-C3 Super Mini, 4MB flash (onboard RX)</t>
   </si>
   <si>
     <t>RISC-V, 2.4GHz WiFi, custom firmware: ESP-NOW RX -&gt; SBUS out (inverted UART) to FC</t>
   </si>
   <si>
-    <t>https://www.aliexpress.com/item/1005005319963906.html</t>
-  </si>
-  <si>
-    <t>Estimated - real AliExpress listings found, $3.50-4.80 USD range</t>
-  </si>
-  <si>
-    <t>ESP32-WROOM-32 DevKit (handheld TX) + KY-023 dual-axis joystick x2 + momentary/toggle switch x2</t>
+    <t>AliExpress (Simple Robot Store)</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005007205044247.html</t>
+  </si>
+  <si>
+    <t>Manufacturer-specified (price/specs from listing, 590 reviews/10,000+ sold, one review confirms board-to-board wireless comms testing); a minority of reviews report WiFi not working out of the box, worth bench-testing WiFi/ESP-NOW range early (Test 5) rather than assuming it works</t>
+  </si>
+  <si>
+    <t>ESP32-WROOM-32 DevKitC (handheld TX) + KY-023 dual-axis joystick x2 + momentary/toggle switch x2</t>
   </si>
   <si>
     <t>Dual-core, 2.4GHz WiFi, custom firmware: reads sticks/switches -&gt; ESP-NOW out. 4 stick axes (throttle, yaw, pitch, roll) + 2 AUX switches (arm, payload release). Powered via USB power bank, already owned, not priced separately.</t>
   </si>
   <si>
-    <t>AliExpress (DevKit $2.20 + 2x joystick $0.60 + 2x switch ~$0.50 est.)</t>
-  </si>
-  <si>
-    <t>https://www.aliexpress.com/item/1005003145871431.html ; https://www.aliexpress.com/item/1882818018.html</t>
-  </si>
-  <si>
-    <t>Estimated - DevKit and joystick prices from real AliExpress listings found; switch price is a typical-component estimate, no specific listing checked</t>
+    <t>AliExpress (DevKit C$1.40 + 2x joystick $0.60 USD + 2x switch ~$0.50 USD est.)</t>
+  </si>
+  <si>
+    <t>https://www.aliexpress.com/item/1005008806241325.html ; https://www.aliexpress.com/item/1882818018.html</t>
+  </si>
+  <si>
+    <t>Manufacturer-specified (DevKit price/specs from listing, 4.9 stars/32 reviews); joystick price from a real AliExpress listing found; switch price is a typical-component estimate, no specific listing checked</t>
   </si>
   <si>
     <t>Motors</t>
@@ -813,13 +816,13 @@
         <v>24</v>
       </c>
       <c r="E3" s="1">
-        <v>5.55</v>
+        <v>1.68</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="G3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="H3" t="s">
         <v>17</v>
@@ -834,7 +837,7 @@
         <v>20</v>
       </c>
       <c r="L3" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -842,22 +845,22 @@
         <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C4">
         <v>1</v>
       </c>
       <c r="D4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E4" s="1">
-        <v>6.12</v>
+        <v>4.46</v>
       </c>
       <c r="F4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="G4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="H4" t="s">
         <v>17</v>
@@ -872,30 +875,30 @@
         <v>20</v>
       </c>
       <c r="L4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E5" s="1">
         <v>33.58</v>
       </c>
       <c r="F5" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H5" t="s">
         <v>17</v>
@@ -910,30 +913,30 @@
         <v>20</v>
       </c>
       <c r="L5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C6">
         <v>1</v>
       </c>
       <c r="D6" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E6" s="1">
         <v>6.24</v>
       </c>
       <c r="F6" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="G6" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="H6" t="s">
         <v>17</v>
@@ -953,28 +956,28 @@
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B7" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C7">
         <v>1</v>
       </c>
       <c r="D7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E7" s="1">
         <v>8.33</v>
       </c>
       <c r="F7" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="G7" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="H7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I7" t="s">
         <v>18</v>
@@ -986,30 +989,30 @@
         <v>20</v>
       </c>
       <c r="L7" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="B8" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C8">
         <v>1</v>
       </c>
       <c r="D8" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E8" s="1">
         <v>4.17</v>
       </c>
       <c r="F8" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="G8" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="H8" t="s">
         <v>17</v>
@@ -1029,25 +1032,25 @@
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C9">
         <v>1</v>
       </c>
       <c r="D9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E9" s="1">
         <v>6</v>
       </c>
       <c r="F9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H9" t="s">
         <v>17</v>
@@ -1062,30 +1065,30 @@
         <v>20</v>
       </c>
       <c r="L9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B10" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="C10">
         <v>1</v>
       </c>
       <c r="D10" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E10" s="1">
         <v>2</v>
       </c>
       <c r="F10" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G10" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H10" t="s">
         <v>17</v>
@@ -1100,33 +1103,33 @@
         <v>20</v>
       </c>
       <c r="L10" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="11" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C11">
         <v>1</v>
       </c>
       <c r="D11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E11" s="1">
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H11" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I11" t="s">
         <v>18</v>
@@ -1138,33 +1141,33 @@
         <v>20</v>
       </c>
       <c r="L11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="12" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="B12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C12">
         <v>1</v>
       </c>
       <c r="D12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E12" s="1">
         <v>4</v>
       </c>
       <c r="F12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="G12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H12" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I12" t="s">
         <v>18</v>
@@ -1173,80 +1176,80 @@
         <v>19</v>
       </c>
       <c r="K12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="L12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="13" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C13">
         <v>1</v>
       </c>
       <c r="D13" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E13" s="1">
         <v>12.51</v>
       </c>
       <c r="F13" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="G13" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="H13" t="s">
         <v>17</v>
       </c>
       <c r="I13" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J13" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K13" t="s">
         <v>20</v>
       </c>
       <c r="L13" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="14" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B14" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C14">
         <v>1</v>
       </c>
       <c r="D14" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E14" s="1">
         <v>59.76</v>
       </c>
       <c r="F14" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="G14" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="H14" t="s">
         <v>17</v>
       </c>
       <c r="I14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J14" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="K14" t="s">
         <v>20</v>
@@ -1257,25 +1260,25 @@
     </row>
     <row r="15" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B15" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C15">
         <v>1</v>
       </c>
       <c r="D15" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E15" s="1">
         <v>33.58</v>
       </c>
       <c r="F15" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G15" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H15" t="s">
         <v>17</v>
@@ -1284,7 +1287,7 @@
         <v>17</v>
       </c>
       <c r="J15" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K15" t="s">
         <v>20</v>
@@ -1295,25 +1298,25 @@
     </row>
     <row r="16" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="B16" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C16">
         <v>1</v>
       </c>
       <c r="D16" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E16" s="1">
         <v>8.33</v>
       </c>
       <c r="F16" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G16" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H16" t="s">
         <v>17</v>
@@ -1322,7 +1325,7 @@
         <v>17</v>
       </c>
       <c r="J16" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K16" t="s">
         <v>20</v>
@@ -1333,107 +1336,107 @@
     </row>
     <row r="17" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B17" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C17">
         <v>1</v>
       </c>
       <c r="D17" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E17" s="1">
         <v>12</v>
       </c>
       <c r="F17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I17" t="s">
         <v>17</v>
       </c>
       <c r="J17" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K17" t="s">
         <v>20</v>
       </c>
       <c r="L17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="18" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B18" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C18">
         <v>1</v>
       </c>
       <c r="D18" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E18" s="1">
         <v>35</v>
       </c>
       <c r="F18" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G18" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="H18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="I18" t="s">
         <v>17</v>
       </c>
       <c r="J18" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K18" t="s">
         <v>20</v>
       </c>
       <c r="L18" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
     <row r="20" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E20" s="5">
-        <v>124.68</v>
+        <v>119.15</v>
       </c>
     </row>
     <row r="21" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E21" s="5">
-        <v>117.95</v>
+        <v>112.42</v>
       </c>
     </row>
     <row r="22" spans="1:5" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E22" s="5">
-        <v>206.86</v>
+        <v>201.33</v>
       </c>
     </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>

</xml_diff>